<commit_message>
asset import system added
</commit_message>
<xml_diff>
--- a/public/import-samples/import-asset.xlsx
+++ b/public/import-samples/import-asset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\laragon-8-3\www\REMARK-OFFICE\asset-management-remark\public\import-samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\asset-management-remark\public\import-samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAC8BEB-F969-42ED-AC46-F41D82B356E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ECE268-8E05-48E7-B5DB-C2D36428820C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="888" yWindow="3360" windowWidth="21048" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Asset Category</t>
   </si>
@@ -46,13 +46,22 @@
   </si>
   <si>
     <t>Store Name</t>
+  </si>
+  <si>
+    <t>Bill Board</t>
+  </si>
+  <si>
+    <t>BIL-STR082-5</t>
+  </si>
+  <si>
+    <t>Kustia Salman Enterprise</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,6 +73,19 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF031B4E"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF031B4E"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -89,9 +111,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -372,16 +396,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" customWidth="1"/>
-    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -402,6 +426,29 @@
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
* kv files code add *kv files validation according to kv * asset type code + double side option add
</commit_message>
<xml_diff>
--- a/public/import-samples/import-asset.xlsx
+++ b/public/import-samples/import-asset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\asset-management-remark\public\import-samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Remark HB\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ECE268-8E05-48E7-B5DB-C2D36428820C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1399EF33-C86D-48CF-BE81-51D1C12B8C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1785" yWindow="5385" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>Asset Category</t>
   </si>
   <si>
-    <t>Asset Name</t>
-  </si>
-  <si>
     <t>Has KV Slot</t>
   </si>
   <si>
@@ -48,20 +45,20 @@
     <t>Store Name</t>
   </si>
   <si>
+    <t>Kustia Salman Enterprise</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
     <t>Bill Board</t>
-  </si>
-  <si>
-    <t>BIL-STR082-5</t>
-  </si>
-  <si>
-    <t>Kustia Salman Enterprise</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,13 +79,6 @@
       <color rgb="FF031B4E"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF031B4E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -111,11 +101,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -396,24 +385,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="33.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -424,36 +413,33 @@
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
+    <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="B3" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation showInputMessage="1" showErrorMessage="1" promptTitle="common asset" sqref="E2:E82" xr:uid="{586F7AA8-B751-4CE4-858A-DE7AF9A8D7AD}"/>
+    <dataValidation showInputMessage="1" showErrorMessage="1" promptTitle="common asset" sqref="D2:D82" xr:uid="{586F7AA8-B751-4CE4-858A-DE7AF9A8D7AD}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>